<commit_message>
scan: seg8 2026-10-10 00:11 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq0_2026-10-08.xlsx
+++ b/output/full_scan/batch_seq0_2026-10-08.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>68.75088630194595</v>
+        <v>68.75088632935142</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>28.10480802837484</v>
+        <v>28.10480798345204</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>3.116797984523913</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>2.32366342052393</v>
+        <v>2.323663420511919</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>78.06529998048428</v>
+        <v>78.06529995721188</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>29.723726801686</v>
+        <v>29.72372678699149</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>6.348785304834501</v>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>81.79201383293488</v>
+        <v>81.79201376531975</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>26.23343329350317</v>
+        <v>26.23343334335112</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>5.050581260309642</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>4.596009139551478</v>
+        <v>4.596009139912002</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>1086.834794706046</v>
+        <v>1086.834794706047</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>48.6</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>68.88225610974031</v>
+        <v>68.8822564367064</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>12.71477370009238</v>
+        <v>12.71477395958657</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>6.053438558221076</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.1809120752235085</v>
+        <v>0.1809120743822979</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>58.45018457873667</v>
+        <v>58.4501845823948</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>20.14320843718718</v>
+        <v>20.14320835786843</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>2.708240513887385</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>2.546725260635307</v>
+        <v>2.54672526120009</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>65.49247125176757</v>
+        <v>65.49247102716717</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>29.36609422556742</v>
+        <v>29.36609443169234</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>3.527633586080116</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.1320563081430936</v>
+        <v>0.1320563083834411</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
         <v>76.84938281567884</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>31.90821670864898</v>
+        <v>31.90821666487004</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>3.499430075610211</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1.690171765293938</v>
+        <v>1.690171765329985</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>62.63600458498946</v>
+        <v>62.63600467842114</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>15.35174302150767</v>
+        <v>15.35174304901884</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.11718406970062</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.2909560719683808</v>
+        <v>0.2909560719082958</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>913.4823175947614</v>
+        <v>913.482317594761</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>21.4</v>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>68.18608195405631</v>
+        <v>68.18608204862969</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>20.83721276025852</v>
+        <v>20.83721268226257</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.057571107754822</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.1903219129909951</v>
+        <v>0.1903219129188931</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>70.13349679223855</v>
+        <v>70.13349677324454</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>28.70745281351844</v>
+        <v>28.70745277612681</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.4778863829004696</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>34.04661907863557</v>
+        <v>34.04661908188027</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>72.94163909775374</v>
+        <v>72.94163908530838</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>41.41361485522605</v>
+        <v>41.41361492438251</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.6692625531607514</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>2.775680817539896</v>
+        <v>2.775680817479805</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>63.96691404230935</v>
+        <v>63.96691405570155</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>25.18102129205635</v>
+        <v>25.18102130560897</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.963357044455915</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>81.41370497450623</v>
+        <v>81.41370495364987</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>19.53505082383182</v>
+        <v>19.53505080478708</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>6.473611031608359</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.08059675246788819</v>
+        <v>0.0805967524654842</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>59.49662286232611</v>
+        <v>59.49662284323976</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>14.91323117272427</v>
+        <v>14.91323119687558</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.534705958997361</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>1.816588389102366</v>
+        <v>1.816588389186494</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>62.4388972160024</v>
+        <v>62.43889721303237</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>23.22194564865272</v>
+        <v>23.22194581142398</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>2.458606094843628</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.3632003323340169</v>
+        <v>0.3632003322859474</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>70.71997515412083</v>
+        <v>70.71997506794207</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>40.20627999984774</v>
+        <v>40.20627998076891</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.046727163758227</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>1.493546111939554</v>
+        <v>1.493546112083774</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>67.49986155495134</v>
+        <v>67.49986120007276</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>21.69462928795212</v>
+        <v>21.69462928795211</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.7143601124408506</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.07590837969097181</v>
+        <v>0.07590837967895631</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>777.3658025572961</v>
+        <v>777.3658025572965</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>36.2</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>65.64095183501165</v>
+        <v>65.64095171659555</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>31.89755916350121</v>
+        <v>31.8975591871857</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>2.945092476757206</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.3817856753405028</v>
+        <v>0.3817856754366376</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>64.16993954706138</v>
+        <v>64.16993955877308</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>20.51075583973391</v>
+        <v>20.51075586539794</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>2.027136419647595</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.0028493324347198</v>
+        <v>0.0028493324467369</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>722.0710344939591</v>
+        <v>722.0710344939585</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>57.1</v>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>61.87037167701789</v>
+        <v>61.87037084885841</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>23.26564229588845</v>
+        <v>23.26564275524422</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.7971046390887576</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>0.4582647886122225</v>
+        <v>0.4582647914963733</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>54.63505011888225</v>
+        <v>54.63505010454895</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>5.317508232370102</v>
+        <v>5.317508223301607</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>5.555703376526621</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.1002464076301624</v>
+        <v>0.1002464075868999</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>59.57192608557797</v>
+        <v>59.571926042572</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>15.09701592889266</v>
+        <v>15.09701590845029</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.903903555197908</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>1.633715834449046</v>
+        <v>1.633715834208718</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>655.4345781659791</v>
+        <v>655.4345781659807</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>230</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>57.41382261893338</v>
+        <v>57.41382265442704</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>21.01761265133142</v>
+        <v>21.01761279270637</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.6416039055495474</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>2.612266514993742</v>
+        <v>2.612266514513069</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>653.8829524402263</v>
+        <v>653.8829524402289</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>68</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>68.28773730178901</v>
+        <v>68.28773726678004</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>15.8947929021889</v>
+        <v>15.89479301723955</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>2.922459904062402</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.863253676281051</v>
+        <v>0.8632536763050837</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>55.20473590781823</v>
+        <v>55.20473590534355</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>37.57523380679167</v>
+        <v>37.57523387915548</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.2622878238583767</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.0543360403054329</v>
+        <v>-0.0543360406659547</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>619.9120315310141</v>
+        <v>619.9120315310139</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>2060</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>47.78381090987602</v>
+        <v>47.78381090353461</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>12.5987322285307</v>
+        <v>12.59873225512207</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.6813679857092976</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-6.808955191873824</v>
+        <v>-6.808955194037194</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>612.5266647546071</v>
+        <v>612.5266647546072</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>85.09999999999999</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>49.11929440422172</v>
+        <v>49.11929424679327</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>19.00406645416426</v>
+        <v>19.00406643453842</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>2.064014355832512</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.3928557141328472</v>
+        <v>0.3928557145053897</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>54.47009015855016</v>
+        <v>54.47009007980888</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>38.52500912334865</v>
+        <v>38.52500915954474</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.2039126708344463</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-0.0536524989102179</v>
+        <v>-0.0536524987660113</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>592.9609450057658</v>
+        <v>592.9609450057661</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>50.1</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>55.83982313956914</v>
+        <v>55.83982066102502</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>4.15883751812657</v>
+        <v>4.15883533012968</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.3131403187712136</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.1419729024590614</v>
+        <v>0.1419729164712351</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>55.07556762034065</v>
+        <v>55.07556764206406</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>23.30970629242927</v>
+        <v>23.3097062805568</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.1556558365170188</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.8245204238784813</v>
+        <v>-0.8245204240106787</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>580.6920907104044</v>
+        <v>580.6920907104042</v>
       </c>
       <c r="E33" s="2" t="n">
         <v>19.4</v>
@@ -2195,7 +2195,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>58.98850584969143</v>
+        <v>58.9885059851096</v>
       </c>
       <c r="I33" s="2" t="n">
         <v>28.8338775140695</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.0367323419004866</v>
+        <v>0.0367323414678635</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>573.2361473756329</v>
+        <v>573.236147375629</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>56.5</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>58.74807538178406</v>
+        <v>58.74807517470344</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>22.86551436745738</v>
+        <v>22.86551444506559</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.108350446873547</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.9196934811197246</v>
+        <v>0.9196934815523486</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>561.6707711957353</v>
+        <v>561.6707711957355</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>326.5</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>48.75616725156184</v>
+        <v>48.75616715356639</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>12.04954635460285</v>
+        <v>12.04954637506356</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.6845297377637236</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.2254880767101654</v>
+        <v>0.2254880780320625</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>53.37589158422116</v>
+        <v>53.37589158890111</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>19.95622744640882</v>
+        <v>19.95622732282192</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>1.06436812333298</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.0257830548826195</v>
+        <v>0.0257830548585841</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>53.29672523006876</v>
+        <v>53.29672523712533</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>27.9068990583525</v>
+        <v>27.90689904747592</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.5209096159834906</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.2432142382569972</v>
+        <v>0.2432142382810365</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>47.11262062905258</v>
+        <v>47.11262082691759</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>10.34898960042178</v>
+        <v>10.34898965396156</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.6407564156104073</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.717665441127562</v>
+        <v>-0.717665445814303</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>54.59729309788906</v>
+        <v>54.59729306043662</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>28.0369515793599</v>
+        <v>28.03695161010849</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.3314914356505022</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.1768901601868906</v>
+        <v>-0.1768901602109416</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>57.70629572668711</v>
+        <v>57.70629571501454</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>28.15750577498932</v>
+        <v>28.15750578982357</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.4782481924665126</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.1912227348127948</v>
+        <v>0.1912227348368318</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>64.76987253322193</v>
+        <v>64.76987249929114</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>32.53685413188181</v>
+        <v>32.53685407189788</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.5670663761275974</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.7175200451707395</v>
+        <v>0.7175200454471335</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>65.40637199469262</v>
+        <v>65.40637205357568</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>49.07272363073445</v>
+        <v>49.07272371017118</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.3507565649380665</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>1.505232419359622</v>
+        <v>1.505232417436822</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>52.38533300237361</v>
+        <v>52.38533302618228</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>27.28451893778002</v>
+        <v>27.2845189981397</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.5146268722717706</v>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>515.1378922641563</v>
+        <v>515.1378922641555</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>24.1</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>56.830794914371</v>
+        <v>56.83079497262705</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>13.91453306425982</v>
+        <v>13.91453302973803</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>2.392350724340234</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.1424846873738943</v>
+        <v>0.1424846873378411</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>54.20933332074446</v>
+        <v>54.20933331408137</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>12.78522607080232</v>
+        <v>12.78522607362251</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.171671703038444</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.220507016725546</v>
+        <v>0.2205070166637593</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>47.65076332000302</v>
+        <v>47.65076339807766</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>34.00702985134878</v>
+        <v>34.00702979493215</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.3792983774624572</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-1.895591269792043</v>
+        <v>-1.895591270203962</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>47.42181609444074</v>
+        <v>47.42181613151857</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>30.8976432166122</v>
+        <v>30.89764327166268</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.8821235310731542</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.8736886222309268</v>
+        <v>-0.8736886222068998</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>461.0112710596544</v>
+        <v>461.0112710596541</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>81</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>40.58445084506695</v>
+        <v>40.58445097475696</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>22.48321764170405</v>
+        <v>22.48321767797798</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.5953315198623444</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.3258135906609768</v>
+        <v>-0.3258135916223669</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>460.538957417092</v>
+        <v>460.5389574170919</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>63.4</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>49.26418390999588</v>
+        <v>49.26418322709255</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>17.75820008719286</v>
+        <v>17.75820020223334</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>1.565331861728069</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.2312142095599967</v>
+        <v>0.2312142104011996</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>51.24182341014726</v>
+        <v>51.24182343523906</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>7.409446058844591</v>
+        <v>7.409446110866228</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.4348522983750438</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.8011644501649202</v>
+        <v>0.8011644496842392</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>47.85265698818198</v>
+        <v>47.8526557618142</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>16.90142867001112</v>
+        <v>16.90142896027152</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>1.207241727081338</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.4152180221018553</v>
+        <v>0.4152180272507331</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>51.09471769887392</v>
+        <v>51.09471769204582</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>5.215468956324937</v>
+        <v>5.21546913308271</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>1.061167350748045</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>1.315487352717326</v>
+        <v>1.315487353270122</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>453.378734983228</v>
+        <v>453.3787349832285</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>26.45</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>19.97018239934931</v>
+        <v>19.9701826039015</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>49.04285851443795</v>
+        <v>49.04285846742758</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.606984700735965</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.1275823386673414</v>
+        <v>-0.1275823389557558</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>447.0431000301944</v>
+        <v>447.0431000301941</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>34.4</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>65.5662966628927</v>
+        <v>65.56629660445458</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>33.14428458119747</v>
+        <v>33.14428463553833</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>2.228843037556953</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.6710381744245847</v>
+        <v>0.6710381746769489</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>439.2716921379535</v>
+        <v>439.2716921379541</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>50.5</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>51.64396867004989</v>
+        <v>51.64396872143281</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>17.95076643234812</v>
+        <v>17.9507664993572</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>1.261462616369482</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.1092348924513225</v>
+        <v>0.1092348924753506</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>53.70635728600141</v>
+        <v>53.70635721462754</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>18.66799548297174</v>
+        <v>18.66799556380727</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.7225547931200471</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.4690026349035413</v>
+        <v>0.469002634975646</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>60.25695172624757</v>
+        <v>60.2569514491917</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>27.2311602706</v>
+        <v>27.23115991647269</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.24034330025339</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>48.05622873834169</v>
+        <v>48.056229116221</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>36.87661600599267</v>
+        <v>36.87661603234269</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.4191745087014877</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.0617997258459984</v>
+        <v>-0.0617997259301209</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>414.2031695476912</v>
+        <v>414.2031695476913</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>139</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>52.08418875083346</v>
+        <v>52.0841887599181</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>31.04128221608954</v>
+        <v>31.04128230463137</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.432183151738959</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.2512553510402679</v>
+        <v>-0.2512553515209683</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>410.3640017409354</v>
+        <v>410.3640017409241</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>30.95</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>48.57514128544108</v>
+        <v>48.57514081278838</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>16.00618360180705</v>
+        <v>16.00618376690014</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.6734366827199414</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.082402606448088</v>
+        <v>0.08240260685667571</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>41.87255004124982</v>
+        <v>41.87255004680194</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>31.70957464210655</v>
+        <v>31.70957463374383</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.5161376373223423</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>1.538462846434086</v>
+        <v>1.53846284616971</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>403.2234296852506</v>
+        <v>403.2234296852505</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>12.75</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>51.66410364899698</v>
+        <v>51.66410372268134</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>13.64569296770591</v>
+        <v>13.64569291512223</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>3.650182642688881</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.016754974943874</v>
+        <v>-0.0167549750039606</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>78.68008853777276</v>
+        <v>78.68008848440415</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>37.30805682429794</v>
+        <v>37.30805683877528</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.1808425508974529</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.1343239081888085</v>
+        <v>0.1343239082052847</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>44.94763305541719</v>
+        <v>44.94763311007497</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>20.60234961324448</v>
+        <v>20.60234959844772</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.6610502872841946</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.0228012556361702</v>
+        <v>-0.0228012556481884</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>44.64499201724888</v>
+        <v>44.64499184255664</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>21.39136576494574</v>
+        <v>21.39136585885247</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.5692080331342624</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.3123991656391873</v>
+        <v>0.3123991659035714</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>395.8634049635209</v>
+        <v>395.8634049635208</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>28.2</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>44.90268834399803</v>
+        <v>44.90268837163893</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>19.1453761405531</v>
+        <v>19.14537615931564</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.870816255095116</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.068620610797997</v>
+        <v>0.0686206105644962</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>42.30937054187002</v>
+        <v>42.30937040162757</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>18.9829820197608</v>
+        <v>18.98298206091577</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.9402414291795336</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>5.455581065764903</v>
+        <v>5.455581070812102</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>385.4744141746589</v>
+        <v>385.4744141746588</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>253.5</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>50.85390714794104</v>
+        <v>50.85390712685061</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>8.51251650267225</v>
+        <v>8.512516585072612</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.3401844706912896</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>2.469308960224295</v>
+        <v>2.469308965872451</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>381.883635821929</v>
+        <v>381.8836358219291</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>20.1</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>48.47937300937726</v>
+        <v>48.47937261553872</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>18.189632038254</v>
+        <v>18.18963212281596</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.5895896159336576</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.0076392896313175</v>
+        <v>-0.0076392895351783</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>37.31450991342541</v>
+        <v>37.31451002180922</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>32.27104997860098</v>
+        <v>32.271049915539</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>2.027341329392833</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.06564547922579141</v>
+        <v>-0.065645479466132</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>40.36133842359701</v>
+        <v>40.36133823499912</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>27.1671622292828</v>
+        <v>27.16716222928279</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.5989563875292683</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>1.113482669414593</v>
+        <v>1.11348267037599</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>363.8756244375477</v>
+        <v>363.8756244375475</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>13.5</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>28.91138071499005</v>
+        <v>28.91138077834961</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>27.43463926876743</v>
+        <v>27.43463923083703</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>3.017999211374759</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.07199120157396439</v>
+        <v>-0.07199120153791259</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>8.186849530617351</v>
+        <v>8.186849521093947</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>38.91875935043327</v>
+        <v>38.91875934096507</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.6442186113205489</v>
+        <v>-0.6442186113085318</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>342.2541318927333</v>
+        <v>342.2541318927296</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>0</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>37.93765132727655</v>
+        <v>37.93765132163702</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>10.29191459269391</v>
+        <v>10.29191463382808</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.1481788815458021</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>46.36827816468684</v>
+        <v>46.36827808779955</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>19.82358684480572</v>
+        <v>19.82358680549904</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.6231276079596844</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.08094866985133729</v>
+        <v>0.0809486699085481</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>47.36883121178813</v>
+        <v>47.36883116445309</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>25.76774569806857</v>
+        <v>25.76774563302967</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.4300255712662324</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>54.4546393564756</v>
+        <v>54.45463913456012</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>12.93439385840971</v>
+        <v>12.93439384546284</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.8082742977947626</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.3510327509488143</v>
+        <v>0.3510327512252116</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>325.5823637249029</v>
+        <v>325.5823637249026</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>21.4</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>40.96968395903292</v>
+        <v>40.96968346809786</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>21.66693844372921</v>
+        <v>21.66693878677197</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.6812827466472959</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.0514943742334104</v>
+        <v>0.0514943744857742</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>320.9511533058237</v>
+        <v>320.9511533058239</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>21.2</v>
@@ -4686,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>49.5099278302382</v>
+        <v>49.50992778181669</v>
       </c>
       <c r="I80" s="2" t="n">
         <v>26.70271905232586</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0085524784235318</v>
+        <v>0.008552478315374</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>42.75933847692557</v>
+        <v>42.75933854615619</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>9.960475002199448</v>
+        <v>9.960474977134094</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.6424088091267123</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.07585755166471971</v>
+        <v>0.0758575517248077</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>28.766054956971</v>
+        <v>28.76605488270419</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>36.71697137807788</v>
+        <v>36.71697133547433</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>2.031379645655545</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>39.32970007741113</v>
+        <v>39.32969969026824</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>24.50740289159818</v>
+        <v>24.50740320759468</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>1.020412423518965</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>1.003513191088885</v>
+        <v>1.003513192290621</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>38.6816204483477</v>
+        <v>38.68162119062995</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>17.61005385355298</v>
+        <v>17.61005387047974</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.4077260477119798</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.0648332523656605</v>
+        <v>0.0648332521253112</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>48.61898133368651</v>
+        <v>48.61898132519884</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>17.15197553124404</v>
+        <v>17.15197557328655</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>1.284509031381192</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>2.359339893073635</v>
+        <v>2.359339893049577</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>304.6597532183896</v>
+        <v>304.6597532183895</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>22.85</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>48.18101952296635</v>
+        <v>48.18101951905166</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>5.134452547981376</v>
+        <v>5.134452575093118</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.4527522101787211</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.0670511741577253</v>
+        <v>0.0670511741817592</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>50.03724842008068</v>
+        <v>50.03724835491892</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>34.28269015400027</v>
+        <v>34.28269027645776</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.2737855717988168</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.0067302870493656</v>
+        <v>-0.0067302870012957</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>44.11381566872717</v>
+        <v>44.11381641374432</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>7.975003476572353</v>
+        <v>7.975003368264433</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.6654817331165166</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>51.69482753190201</v>
+        <v>51.69482809709368</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>32.46331487373325</v>
+        <v>32.46332434370365</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.413418222611168</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.1009603142557269</v>
+        <v>0.1009603071775346</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>282.6055382257987</v>
+        <v>282.6055382257988</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>9.65</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>37.30767587746976</v>
+        <v>37.30767331140419</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>26.13846135011506</v>
+        <v>26.13846145517847</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.497673942166656</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.0072446634574273</v>
+        <v>-0.0072446632290987</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>279.1479950597467</v>
+        <v>279.1479950597472</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>58.4</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>16.26069884120197</v>
+        <v>16.26069884838886</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>36.15212986199487</v>
+        <v>36.15212981069186</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.04537194403018</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1743288727172258</v>
+        <v>-0.1743288727652986</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>273.5740563964841</v>
+        <v>273.574056396484</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>15.15</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>53.51978085092245</v>
+        <v>53.51978105138596</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>11.42925392938144</v>
+        <v>11.42925411410283</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.2729448192959408</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.0484213543037463</v>
+        <v>0.0484213541715555</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>273.1714851159183</v>
+        <v>273.1714851159185</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>199.5</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>39.2441181299348</v>
+        <v>39.24411813866484</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>12.94927338308331</v>
+        <v>12.9492733830833</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.020988026920266</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.3233670559437325</v>
+        <v>0.323367055823577</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>47.11690506183617</v>
+        <v>47.1169050348886</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>46.49694560027209</v>
+        <v>46.4969456456187</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.067541341736764</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.1096514112116624</v>
+        <v>0.1096514111635917</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>267.7887244624446</v>
+        <v>267.7887244624445</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>140</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>44.4228761533243</v>
+        <v>44.42287609493049</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>7.523932378013983</v>
+        <v>7.523932393340924</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.199927762321393</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.1314310497029081</v>
+        <v>0.1314310485011802</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>44.61126930798109</v>
+        <v>44.6112693938418</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>52.49667401250918</v>
+        <v>52.49667392345407</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.9088271535977084</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>44.08451299593214</v>
+        <v>44.08451311235183</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>14.27682828410773</v>
+        <v>14.27682831659762</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.5238754844087758</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0373960928947667</v>
+        <v>0.037396092858715</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>247.3526021820107</v>
+        <v>247.3526021820109</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>44.5</v>
@@ -5643,7 +5643,7 @@
         <v>50.27470372235318</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>8.957065075895995</v>
+        <v>8.957065137947493</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>1.113023618742389</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.7257028829608629</v>
+        <v>0.725702883008934</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>47.26365857642308</v>
+        <v>47.26365854264361</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>11.72338521848564</v>
+        <v>11.72338522170471</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4248457621423513</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.6324199211364632</v>
+        <v>0.6324199214969837</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>49.76560314618668</v>
+        <v>49.76560302511928</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>13.65590901646543</v>
+        <v>13.65590902203867</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>1.256252621157641</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.3767863554903351</v>
+        <v>0.3767863556465586</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>240.6094488777084</v>
+        <v>240.6094488777083</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>29.85</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>42.87981992314916</v>
+        <v>42.87981975660852</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>12.6283898921754</v>
+        <v>12.6283900105753</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.7551403039045136</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.07353961685529251</v>
+        <v>0.0735396170235324</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>229.8513971298646</v>
+        <v>229.8513971298647</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>10.3</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>42.34906414883429</v>
+        <v>42.34906423635634</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>16.44365345226704</v>
+        <v>16.44365345752313</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.1301251686168711</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.1209711912520924</v>
+        <v>-0.1209711913602483</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>40.73938009094184</v>
+        <v>40.73937871427032</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>8.79481684222638</v>
+        <v>8.794816886834091</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.3870128060262118</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.1050530017710232</v>
+        <v>0.1050530029246817</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>37.05648657506774</v>
+        <v>37.05648644967242</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>12.61022694312326</v>
+        <v>12.61022695342716</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.7273447076327048</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.029876980103937</v>
+        <v>-0.0298769800799026</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>43.58420405043517</v>
+        <v>43.5842038159188</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>7.421168279513759</v>
+        <v>7.421168319736209</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.4531701565060215</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.005698230775918</v>
+        <v>0.0056982307807249</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>215.5256206284074</v>
+        <v>215.5256206284072</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>40.6</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>44.76596797719962</v>
+        <v>44.7659681387316</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>12.1608071468484</v>
+        <v>12.16080718526336</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.3809097872785837</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.0491573663829944</v>
+        <v>-0.0491573665031703</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>214.9278119846296</v>
+        <v>214.9278119846295</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>40.9</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>53.92689334659694</v>
+        <v>53.92689331764274</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>14.43765889412709</v>
+        <v>14.43765886797527</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>1.045493223751115</v>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>207.2533452155243</v>
+        <v>207.2533452155261</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>39.3</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>46.43233050633585</v>
+        <v>46.4323300759787</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>15.45636345813229</v>
+        <v>15.45636357093937</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.3948254321441044</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.1830199942334583</v>
+        <v>0.1830199946901065</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>40.30402073533084</v>
+        <v>40.30402100914071</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>27.99119920105399</v>
+        <v>27.99119922148739</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.0915954713824829</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-1.15845807655587</v>
+        <v>-1.158458077373055</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>183.6479593256479</v>
+        <v>183.647959325648</v>
       </c>
       <c r="E110" s="2" t="n">
         <v>74.09999999999999</v>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>36.58205565005205</v>
+        <v>36.58205534000025</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>10.15759231702086</v>
+        <v>10.15759242355149</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.391547480317337</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.0670311014749827</v>
+        <v>-0.0670311012346347</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>32.33699037530904</v>
+        <v>32.33699024086408</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.03304013043113</v>
+        <v>17.03304014948704</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.7136039970620186</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.0623463217892638</v>
+        <v>0.0623463218301228</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>50.00508989235949</v>
+        <v>50.00508988237379</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>17.16102169162326</v>
+        <v>17.16102174116885</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.5176419555989005</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1096968622204609</v>
+        <v>0.1096968622444947</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>146.0612632875095</v>
+        <v>146.0612632875094</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>90.90000000000001</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>43.10246644545018</v>
+        <v>43.10246649428943</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>19.73462802626165</v>
+        <v>19.73462790332274</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.9333942982762388</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>42.90424339535345</v>
+        <v>42.90424351613235</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>11.69162783546806</v>
+        <v>11.6916278776238</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.4024438372040744</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0160860633166056</v>
+        <v>0.0160860631002954</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>144.8572864131397</v>
+        <v>144.8572864131396</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>11.5</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>44.57729103507442</v>
+        <v>44.57729662833026</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>17.10783972056232</v>
+        <v>17.10783998825587</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.0983745110757316</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0373666358650294</v>
+        <v>-0.0373666390255794</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>36.37939091386696</v>
+        <v>36.37930077741147</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>5.328014816327801</v>
+        <v>5.327904602012652</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.4352871123868269</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.0430417503419926</v>
+        <v>0.0430368640187484</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>

</xml_diff>